<commit_message>
feat(universe): execute service partition S02
</commit_message>
<xml_diff>
--- a/config/universe-generated/templates/Universe.xlsx
+++ b/config/universe-generated/templates/Universe.xlsx
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1660" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1668" uniqueCount="270">
   <si>
     <t>@table</t>
   </si>
@@ -734,7 +734,13 @@
     <t>UniverseService</t>
   </si>
   <si>
-    <t>cfda7f55bc9d8c98</t>
+    <t>b59e6357048735cf</t>
+  </si>
+  <si>
+    <t>profile_owner</t>
+  </si>
+  <si>
+    <t>source_event_id</t>
   </si>
   <si>
     <t>currency_stable_key</t>
@@ -747,6 +753,12 @@
   </si>
   <si>
     <t>enum&lt;UniverseServiceKind&gt;</t>
+  </si>
+  <si>
+    <t>enum&lt;UniverseServiceProfileOwner&gt;</t>
+  </si>
+  <si>
+    <t>optional&lt;i32&gt;</t>
   </si>
   <si>
     <t>UniverseServiceParameter</t>
@@ -5202,21 +5214,23 @@
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
     <col min="4" max="4" width="25.7109375" style="5" customWidth="1"/>
-    <col min="5" max="5" width="19.7109375" style="5" customWidth="1"/>
-    <col min="6" max="6" width="24.7109375" style="5" customWidth="1"/>
-    <col min="7" max="7" width="21.7109375" style="5" customWidth="1"/>
-    <col min="8" max="8" width="15.7109375" style="5" customWidth="1"/>
-    <col min="9" max="11" width="12.7109375" style="5" customWidth="1"/>
-    <col min="12" max="12" width="13.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="32.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="19.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="24.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="21.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="15.7109375" style="5" customWidth="1"/>
+    <col min="11" max="13" width="12.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="13.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5248,7 +5262,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="24" customHeight="1">
+    <row r="2" spans="1:14" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -5271,22 +5285,28 @@
         <v>232</v>
       </c>
       <c r="H2" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="J2" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="K2" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="L2" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="M2" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:14">
       <c r="A3" s="4" t="s">
         <v>19</v>
       </c>
@@ -5309,22 +5329,28 @@
         <v>232</v>
       </c>
       <c r="H3" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="J3" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="K3" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="L3" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="K3" s="5" t="s">
+      <c r="M3" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="L3" s="5" t="s">
+      <c r="N3" s="5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:14">
       <c r="A4" s="4" t="s">
         <v>20</v>
       </c>
@@ -5335,22 +5361,22 @@
         <v>22</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>60</v>
+        <v>236</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>60</v>
+        <v>237</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>60</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>22</v>
@@ -5361,8 +5387,14 @@
       <c r="L4" s="5" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="5" spans="1:12">
+      <c r="M4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
       <c r="A5" s="4" t="s">
         <v>23</v>
       </c>
@@ -5399,8 +5431,14 @@
       <c r="L5" s="5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:12">
+      <c r="M5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
       <c r="A6" s="4" t="s">
         <v>24</v>
       </c>
@@ -5414,23 +5452,25 @@
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="K6" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="J6" s="5" t="s">
+      <c r="L6" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="K6" s="5" t="s">
+      <c r="M6" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="L6" s="5" t="s">
+      <c r="N6" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="42" customHeight="1">
+    <row r="7" spans="1:14" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>32</v>
       </c>
@@ -5445,15 +5485,20 @@
       <c r="J7" s="6"/>
       <c r="K7" s="6"/>
       <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Currency, ResetBlessing, Reviver, Downloader, RespiteOffers, EnhanceBlessing, BlessingShop, CurioShop, TrailblazeBonus" promptTitle="UniverseServiceKind enum" prompt="Select a value from the dropdown." sqref="D8:D1007">
       <formula1>"Currency,ResetBlessing,Reviver,Downloader,RespiteOffers,EnhanceBlessing,BlessingShop,CurioShop,TrailblazeBonus"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Standard, SwarmDisaster, GoldAndGears, DivergentUniverse" promptTitle="UniverseServiceProfileOwner enum" prompt="Select a value from the dropdown." sqref="E8:E1007">
+      <formula1>"Standard,SwarmDisaster,GoldAndGears,DivergentUniverse"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5475,7 +5520,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5497,7 +5542,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -5505,16 +5550,16 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -5522,16 +5567,16 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -5539,7 +5584,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -5624,7 +5669,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5648,7 +5693,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="24" customHeight="1">
@@ -5662,19 +5707,19 @@
         <v>11</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>135</v>
@@ -5703,19 +5748,19 @@
         <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>135</v>
@@ -5747,7 +5792,7 @@
         <v>84</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>22</v>
@@ -5902,7 +5947,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5924,7 +5969,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -5932,13 +5977,13 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -5946,13 +5991,13 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -5960,13 +6005,13 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -6282,7 +6327,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -6304,7 +6349,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -6312,16 +6357,16 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -6329,16 +6374,16 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -6346,7 +6391,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -6430,7 +6475,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -6452,7 +6497,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -6460,7 +6505,7 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
@@ -6469,16 +6514,16 @@
         <v>52</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>143</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -6486,7 +6531,7 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
@@ -6495,16 +6540,16 @@
         <v>52</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>143</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -6512,13 +6557,13 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>22</v>
@@ -6527,7 +6572,7 @@
         <v>22</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>60</v>
@@ -6622,7 +6667,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -6644,7 +6689,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -6652,7 +6697,7 @@
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>69</v>
@@ -6666,7 +6711,7 @@
         <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>69</v>
@@ -6680,7 +6725,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>

</xml_diff>